<commit_message>
Main Module with data driven working
</commit_message>
<xml_diff>
--- a/mvn-project/src/test/resources/testdata/purnatestdata.xlsx
+++ b/mvn-project/src/test/resources/testdata/purnatestdata.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abhishek\eclipse-workspace\mvn-project\src\test\resources\testdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abhishek\git\mvn-project\mvn-project\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7755" activeTab="4"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7755" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="customer" sheetId="1" r:id="rId1"/>
@@ -366,24 +366,12 @@
     <t>40</t>
   </si>
   <si>
-    <t>06112022</t>
-  </si>
-  <si>
-    <t>04052022</t>
-  </si>
-  <si>
     <t>3</t>
   </si>
   <si>
     <t>4</t>
   </si>
   <si>
-    <t>02082022</t>
-  </si>
-  <si>
-    <t>04042022</t>
-  </si>
-  <si>
     <t>4040404040</t>
   </si>
   <si>
@@ -1057,6 +1045,18 @@
   </si>
   <si>
     <t>9</t>
+  </si>
+  <si>
+    <t>04022021</t>
+  </si>
+  <si>
+    <t>03062020</t>
+  </si>
+  <si>
+    <t>01012022</t>
+  </si>
+  <si>
+    <t>09092019</t>
   </si>
 </sst>
 </file>
@@ -1123,9 +1123,9 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1464,7 +1464,7 @@
         <v>9</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>10</v>
@@ -1479,7 +1479,7 @@
         <v>12</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>13</v>
@@ -1499,7 +1499,7 @@
         <v>18</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>19</v>
@@ -1514,7 +1514,7 @@
         <v>21</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>22</v>
@@ -1528,13 +1528,13 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>25</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>26</v>
@@ -1549,7 +1549,7 @@
         <v>28</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>29</v>
@@ -1562,38 +1562,38 @@
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
-        <v>115</v>
+      <c r="A5" s="6" t="s">
+        <v>113</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="H5" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="I5" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="E5" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="F5" s="2" t="s">
+      <c r="J5" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="K5" s="2" t="s">
         <v>138</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>139</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="K5" s="2" t="s">
-        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -1626,37 +1626,37 @@
         <v>92</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="H1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>147</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -1664,28 +1664,28 @@
         <v>102</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="G2" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="H2" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="E2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>156</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>158</v>
-      </c>
-      <c r="H2" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>160</v>
       </c>
       <c r="J2" s="5" t="s">
         <v>103</v>
@@ -1694,7 +1694,7 @@
         <v>103</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
@@ -1702,113 +1702,113 @@
         <v>103</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="F3" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="G3" s="5" t="s">
         <v>163</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>167</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>103</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="G4" s="6" t="s">
         <v>171</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="H4" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="J4" s="6" t="s">
         <v>172</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="K4" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="L4" s="6" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="I5" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="E4" s="8" t="s">
-        <v>173</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>174</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>175</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>114</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="J4" s="7" t="s">
-        <v>176</v>
-      </c>
-      <c r="K4" s="7" t="s">
-        <v>177</v>
-      </c>
-      <c r="L4" s="7" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
-        <v>115</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="E5" s="8" t="s">
+      <c r="J5" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="F5" s="7" t="s">
-        <v>182</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>183</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>184</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="J5" s="7" t="s">
-        <v>185</v>
-      </c>
-      <c r="K5" s="7" t="s">
+      <c r="K5" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="L5" s="7" t="s">
-        <v>157</v>
+      <c r="L5" s="6" t="s">
+        <v>153</v>
       </c>
     </row>
   </sheetData>
@@ -1830,16 +1830,16 @@
         <v>92</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>1</v>
@@ -1847,19 +1847,19 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>9</v>
@@ -1867,39 +1867,39 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>25</v>
@@ -1907,19 +1907,19 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="E5" s="5" t="s">
         <v>204</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>208</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>18</v>
@@ -2034,8 +2034,8 @@
       <c r="B2" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C2" s="6" t="s">
-        <v>112</v>
+      <c r="C2" s="4" t="s">
+        <v>341</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>46</v>
@@ -2102,8 +2102,8 @@
       <c r="B3" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C3" s="6" t="s">
-        <v>113</v>
+      <c r="C3" s="4" t="s">
+        <v>339</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>46</v>
@@ -2165,13 +2165,13 @@
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C4" s="6" t="s">
-        <v>116</v>
+      <c r="C4" s="8" t="s">
+        <v>340</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>68</v>
@@ -2180,10 +2180,10 @@
         <v>69</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>70</v>
@@ -2219,27 +2219,27 @@
         <v>74</v>
       </c>
       <c r="S4" s="5" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="T4" s="2" t="s">
         <v>77</v>
       </c>
       <c r="U4" s="5" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="V4" s="5" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="C5" s="6" t="s">
-        <v>117</v>
+      <c r="C5" s="8" t="s">
+        <v>342</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>46</v>
@@ -2248,10 +2248,10 @@
         <v>79</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>80</v>
@@ -2287,16 +2287,16 @@
         <v>84</v>
       </c>
       <c r="S5" s="5" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="T5" s="2" t="s">
         <v>91</v>
       </c>
       <c r="U5" s="5" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="V5" s="5" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -2311,7 +2311,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="22.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="31.5703125" bestFit="1" customWidth="1"/>
@@ -2328,43 +2328,43 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>248</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>249</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>250</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>251</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -2372,40 +2372,40 @@
         <v>102</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="I2" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="J2" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="K2" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="L2" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="M2" s="2" t="s">
         <v>211</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>216</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>270</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>224</v>
-      </c>
-      <c r="L2" s="5" t="s">
-        <v>225</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -2413,368 +2413,368 @@
         <v>103</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="F3" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="G3" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="F3" s="2" t="s">
+      <c r="H3" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="L3" s="5" t="s">
         <v>222</v>
       </c>
-      <c r="G3" s="5" t="s">
-        <v>223</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>271</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>275</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="L3" s="5" t="s">
-        <v>226</v>
-      </c>
       <c r="M3" s="2" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="G4" s="5" t="s">
         <v>230</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="H4" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="I4" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="J4" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="K4" s="2" t="s">
         <v>233</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="L4" s="5" t="s">
         <v>234</v>
       </c>
-      <c r="H4" s="2" t="s">
-        <v>272</v>
-      </c>
-      <c r="I4" s="2" t="s">
+      <c r="M4" s="2" t="s">
         <v>235</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>236</v>
-      </c>
-      <c r="K4" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="L4" s="5" t="s">
-        <v>238</v>
-      </c>
-      <c r="M4" s="2" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="B5" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>251</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="F5" s="7" t="s">
         <v>253</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="G5" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>269</v>
+      </c>
+      <c r="I5" s="7" t="s">
         <v>254</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="J5" s="7" t="s">
         <v>255</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="K5" s="7" t="s">
         <v>256</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="L5" s="6" t="s">
         <v>257</v>
       </c>
-      <c r="G5" s="7" t="s">
-        <v>268</v>
-      </c>
-      <c r="H5" s="8" t="s">
-        <v>273</v>
-      </c>
-      <c r="I5" s="8" t="s">
+      <c r="M5" s="7" t="s">
         <v>258</v>
-      </c>
-      <c r="J5" s="8" t="s">
-        <v>259</v>
-      </c>
-      <c r="K5" s="8" t="s">
-        <v>260</v>
-      </c>
-      <c r="L5" s="7" t="s">
-        <v>261</v>
-      </c>
-      <c r="M5" s="8" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="B6" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>259</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>261</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="F6" s="7" t="s">
         <v>263</v>
       </c>
-      <c r="C6" s="5" t="s">
-        <v>264</v>
-      </c>
-      <c r="D6" s="8" t="s">
+      <c r="G6" s="6" t="s">
         <v>265</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>266</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>267</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>269</v>
-      </c>
-      <c r="H6" s="8" t="s">
+      <c r="H6" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>273</v>
+      </c>
+      <c r="K6" s="7" t="s">
         <v>274</v>
       </c>
-      <c r="I6" s="8" t="s">
+      <c r="L6" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="M6" s="7" t="s">
         <v>276</v>
-      </c>
-      <c r="J6" s="8" t="s">
-        <v>277</v>
-      </c>
-      <c r="K6" s="8" t="s">
-        <v>278</v>
-      </c>
-      <c r="L6" s="7" t="s">
-        <v>279</v>
-      </c>
-      <c r="M6" s="8" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="B7" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>279</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="F7" s="7" t="s">
         <v>281</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="G7" s="6" t="s">
         <v>282</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="H7" s="7" t="s">
         <v>283</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="I7" s="7" t="s">
         <v>284</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="J7" s="7" t="s">
         <v>285</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="K7" s="7" t="s">
         <v>286</v>
       </c>
-      <c r="H7" s="8" t="s">
+      <c r="L7" s="6" t="s">
         <v>287</v>
       </c>
-      <c r="I7" s="8" t="s">
-        <v>288</v>
-      </c>
-      <c r="J7" s="8" t="s">
-        <v>289</v>
-      </c>
-      <c r="K7" s="8" t="s">
-        <v>290</v>
-      </c>
-      <c r="L7" s="7" t="s">
-        <v>291</v>
-      </c>
-      <c r="M7" s="8" t="s">
-        <v>304</v>
+      <c r="M7" s="7" t="s">
+        <v>300</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>198</v>
-      </c>
-      <c r="B8" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>288</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>290</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="F8" s="7" t="s">
         <v>292</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="G8" s="6" t="s">
         <v>293</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="H8" s="7" t="s">
         <v>294</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="I8" s="7" t="s">
         <v>295</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="J8" s="7" t="s">
         <v>296</v>
       </c>
-      <c r="G8" s="7" t="s">
+      <c r="K8" s="7" t="s">
         <v>297</v>
       </c>
-      <c r="H8" s="8" t="s">
+      <c r="L8" s="6" t="s">
         <v>298</v>
       </c>
-      <c r="I8" s="8" t="s">
+      <c r="M8" s="7" t="s">
         <v>299</v>
-      </c>
-      <c r="J8" s="8" t="s">
-        <v>300</v>
-      </c>
-      <c r="K8" s="8" t="s">
-        <v>301</v>
-      </c>
-      <c r="L8" s="7" t="s">
-        <v>302</v>
-      </c>
-      <c r="M8" s="8" t="s">
-        <v>303</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>202</v>
-      </c>
-      <c r="B9" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>302</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>303</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="F9" s="7" t="s">
         <v>305</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="G9" s="6" t="s">
         <v>306</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="H9" s="7" t="s">
         <v>307</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="I9" s="7" t="s">
         <v>308</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="J9" s="7" t="s">
         <v>309</v>
       </c>
-      <c r="G9" s="7" t="s">
+      <c r="K9" s="7" t="s">
         <v>310</v>
       </c>
-      <c r="H9" s="8" t="s">
+      <c r="L9" s="6" t="s">
         <v>311</v>
       </c>
-      <c r="I9" s="8" t="s">
+      <c r="M9" s="7" t="s">
         <v>312</v>
-      </c>
-      <c r="J9" s="8" t="s">
-        <v>313</v>
-      </c>
-      <c r="K9" s="8" t="s">
-        <v>314</v>
-      </c>
-      <c r="L9" s="7" t="s">
-        <v>315</v>
-      </c>
-      <c r="M9" s="8" t="s">
-        <v>316</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>342</v>
-      </c>
-      <c r="B10" s="8" t="s">
+        <v>338</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>313</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>314</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>315</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="F10" s="7" t="s">
         <v>317</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="G10" s="6" t="s">
         <v>318</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="H10" s="7" t="s">
         <v>319</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="I10" s="7" t="s">
         <v>320</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="J10" s="7" t="s">
         <v>321</v>
       </c>
-      <c r="G10" s="7" t="s">
+      <c r="K10" s="7" t="s">
         <v>322</v>
       </c>
-      <c r="H10" s="8" t="s">
+      <c r="L10" s="6" t="s">
         <v>323</v>
       </c>
-      <c r="I10" s="8" t="s">
+      <c r="M10" s="7" t="s">
         <v>324</v>
-      </c>
-      <c r="J10" s="8" t="s">
-        <v>325</v>
-      </c>
-      <c r="K10" s="8" t="s">
-        <v>326</v>
-      </c>
-      <c r="L10" s="7" t="s">
-        <v>327</v>
-      </c>
-      <c r="M10" s="8" t="s">
-        <v>328</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="B11" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>325</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>326</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>327</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="F11" s="7" t="s">
         <v>329</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="G11" s="6" t="s">
         <v>330</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="H11" s="7" t="s">
         <v>331</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="I11" s="7" t="s">
         <v>332</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="J11" s="7" t="s">
         <v>333</v>
       </c>
-      <c r="G11" s="7" t="s">
+      <c r="K11" s="7" t="s">
         <v>334</v>
       </c>
-      <c r="H11" s="8" t="s">
+      <c r="L11" s="6" t="s">
         <v>335</v>
       </c>
-      <c r="I11" s="8" t="s">
+      <c r="M11" s="7" t="s">
         <v>336</v>
-      </c>
-      <c r="J11" s="8" t="s">
-        <v>337</v>
-      </c>
-      <c r="K11" s="8" t="s">
-        <v>338</v>
-      </c>
-      <c r="L11" s="7" t="s">
-        <v>339</v>
-      </c>
-      <c r="M11" s="8" t="s">
-        <v>340</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added to local git
</commit_message>
<xml_diff>
--- a/mvn-project/src/test/resources/testdata/purnatestdata.xlsx
+++ b/mvn-project/src/test/resources/testdata/purnatestdata.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7755" activeTab="3"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7755"/>
   </bookViews>
   <sheets>
     <sheet name="customer" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="343">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="346">
   <si>
     <t>CUSTOMER_NO</t>
   </si>
@@ -165,27 +165,12 @@
     <t>NO_OF_DAYS</t>
   </si>
   <si>
-    <t>arun</t>
-  </si>
-  <si>
-    <t>purchases</t>
-  </si>
-  <si>
-    <t>jr. purchase assistant</t>
-  </si>
-  <si>
     <t>arun_pan_no_123</t>
   </si>
   <si>
     <t>arun@gmail.com</t>
   </si>
   <si>
-    <t>gandhi nagar</t>
-  </si>
-  <si>
-    <t>pune</t>
-  </si>
-  <si>
     <t>AB+</t>
   </si>
   <si>
@@ -198,21 +183,12 @@
     <t>ABC025480</t>
   </si>
   <si>
-    <t>dilip</t>
-  </si>
-  <si>
-    <t>purchase assistant</t>
-  </si>
-  <si>
     <t>dilip_pan_no_852</t>
   </si>
   <si>
     <t>dilip@gmail.com</t>
   </si>
   <si>
-    <t>laxmi nagar</t>
-  </si>
-  <si>
     <t>B+</t>
   </si>
   <si>
@@ -231,24 +207,12 @@
     <t>AXIS81067</t>
   </si>
   <si>
-    <t>suraj</t>
-  </si>
-  <si>
-    <t>sales</t>
-  </si>
-  <si>
-    <t>jr. sales assistant</t>
-  </si>
-  <si>
     <t>suraj_pan_no_630</t>
   </si>
   <si>
     <t>suraj@gmail.com</t>
   </si>
   <si>
-    <t>karve nagar</t>
-  </si>
-  <si>
     <t>O+</t>
   </si>
   <si>
@@ -264,21 +228,12 @@
     <t>SBI60483</t>
   </si>
   <si>
-    <t>karan</t>
-  </si>
-  <si>
-    <t>manager</t>
-  </si>
-  <si>
     <t>karan_pan_no_787</t>
   </si>
   <si>
     <t>karan@gmail.com</t>
   </si>
   <si>
-    <t>station road</t>
-  </si>
-  <si>
     <t>A+</t>
   </si>
   <si>
@@ -426,9 +381,6 @@
     <t>8800648234</t>
   </si>
   <si>
-    <t>lane no 9 sector no 10 norht road pune</t>
-  </si>
-  <si>
     <t>customer_4@gmail.com</t>
   </si>
   <si>
@@ -1057,6 +1009,63 @@
   </si>
   <si>
     <t>09092019</t>
+  </si>
+  <si>
+    <t>Arun</t>
+  </si>
+  <si>
+    <t>Dilip</t>
+  </si>
+  <si>
+    <t>Suraj</t>
+  </si>
+  <si>
+    <t>Karan</t>
+  </si>
+  <si>
+    <t>Purchases</t>
+  </si>
+  <si>
+    <t>Sales</t>
+  </si>
+  <si>
+    <t>Jr. Purchase Assistant</t>
+  </si>
+  <si>
+    <t>Purchase Assistant</t>
+  </si>
+  <si>
+    <t>Jr. Sales Assistant</t>
+  </si>
+  <si>
+    <t>Manager</t>
+  </si>
+  <si>
+    <t>Gandhi Nagar Pune</t>
+  </si>
+  <si>
+    <t>Laxmi Nagar Pune</t>
+  </si>
+  <si>
+    <t>Station Road Pune</t>
+  </si>
+  <si>
+    <t>Gandhi Nagar</t>
+  </si>
+  <si>
+    <t>Laxmi Nagar</t>
+  </si>
+  <si>
+    <t>Karve Nagar</t>
+  </si>
+  <si>
+    <t>Station Road</t>
+  </si>
+  <si>
+    <t>Pune</t>
+  </si>
+  <si>
+    <t>lane no 9 sector no 10 north road pune</t>
   </si>
 </sst>
 </file>
@@ -1458,13 +1467,13 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>102</v>
+        <v>87</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>124</v>
+        <v>109</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>10</v>
@@ -1479,7 +1488,7 @@
         <v>12</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>127</v>
+        <v>112</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>13</v>
@@ -1493,13 +1502,13 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>103</v>
+        <v>88</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>18</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>125</v>
+        <v>110</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>19</v>
@@ -1514,7 +1523,7 @@
         <v>21</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>128</v>
+        <v>113</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>22</v>
@@ -1528,13 +1537,13 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>112</v>
+        <v>97</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>25</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>126</v>
+        <v>111</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>26</v>
@@ -1549,7 +1558,7 @@
         <v>28</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>129</v>
+        <v>114</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>29</v>
@@ -1563,37 +1572,37 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>113</v>
+        <v>98</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>130</v>
+        <v>115</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>132</v>
+        <v>345</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>132</v>
+        <v>345</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>133</v>
+        <v>117</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>134</v>
+        <v>118</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>135</v>
+        <v>119</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>136</v>
+        <v>120</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>137</v>
+        <v>121</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>138</v>
+        <v>122</v>
       </c>
     </row>
   </sheetData>
@@ -1623,192 +1632,192 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>139</v>
+        <v>123</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>140</v>
+        <v>124</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>141</v>
+        <v>125</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>142</v>
+        <v>126</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>148</v>
+        <v>132</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>149</v>
+        <v>133</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>143</v>
+        <v>127</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>144</v>
+        <v>128</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>145</v>
+        <v>129</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>146</v>
+        <v>130</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>147</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>102</v>
+        <v>87</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>166</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>152</v>
+        <v>136</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>153</v>
+        <v>137</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>154</v>
+        <v>138</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>155</v>
+        <v>139</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>156</v>
+        <v>140</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>103</v>
+        <v>88</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>103</v>
+        <v>88</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>157</v>
+        <v>141</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>103</v>
+        <v>88</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>158</v>
+        <v>142</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>159</v>
+        <v>143</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>161</v>
+        <v>145</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>162</v>
+        <v>146</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>163</v>
+        <v>147</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>103</v>
+        <v>88</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>164</v>
+        <v>148</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>165</v>
+        <v>149</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>112</v>
+        <v>97</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>122</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>112</v>
+        <v>97</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>167</v>
+        <v>151</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>168</v>
+        <v>152</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>169</v>
+        <v>153</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>170</v>
+        <v>154</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>171</v>
+        <v>155</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>112</v>
+        <v>97</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>164</v>
+        <v>148</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>172</v>
+        <v>156</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>173</v>
+        <v>157</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>174</v>
+        <v>158</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>113</v>
+        <v>98</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>175</v>
+        <v>159</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>176</v>
+        <v>160</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>177</v>
+        <v>161</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>178</v>
+        <v>162</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>179</v>
+        <v>163</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>180</v>
+        <v>164</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>164</v>
+        <v>148</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>181</v>
+        <v>165</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>103</v>
+        <v>88</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>153</v>
+        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -1827,19 +1836,19 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>182</v>
+        <v>166</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>183</v>
+        <v>167</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>184</v>
+        <v>168</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>185</v>
+        <v>169</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>1</v>
@@ -1847,19 +1856,19 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>180</v>
+        <v>164</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>187</v>
+        <v>171</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>186</v>
+        <v>170</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>188</v>
+        <v>172</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>189</v>
+        <v>173</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>9</v>
@@ -1867,39 +1876,39 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>190</v>
+        <v>174</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>191</v>
+        <v>175</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>192</v>
+        <v>176</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>201</v>
+        <v>185</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>193</v>
+        <v>177</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>130</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>194</v>
+        <v>178</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>195</v>
+        <v>179</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>196</v>
+        <v>180</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>202</v>
+        <v>186</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>197</v>
+        <v>181</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>25</v>
@@ -1907,19 +1916,19 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>198</v>
+        <v>182</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>200</v>
+        <v>184</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>199</v>
+        <v>183</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>203</v>
+        <v>187</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>204</v>
+        <v>188</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>18</v>
@@ -1939,21 +1948,21 @@
     <col min="2" max="2" width="6.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="17.7109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.85546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.140625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="9" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="12.42578125" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="7.5703125" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="12.85546875" bestFit="1" customWidth="1"/>
@@ -1961,13 +1970,13 @@
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>32</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>33</v>
@@ -1979,7 +1988,7 @@
         <v>35</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>7</v>
@@ -2006,19 +2015,19 @@
         <v>42</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>97</v>
+        <v>82</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>98</v>
+        <v>83</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>99</v>
+        <v>84</v>
       </c>
       <c r="U1" s="1" t="s">
         <v>43</v>
@@ -2029,274 +2038,274 @@
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>102</v>
+        <v>87</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>341</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>49</v>
-      </c>
       <c r="J2" s="2" t="s">
-        <v>50</v>
+        <v>340</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>51</v>
+        <v>344</v>
       </c>
       <c r="L2" s="3">
         <v>33197</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>53</v>
+        <v>337</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="P2" s="2" t="s">
-        <v>89</v>
+        <v>74</v>
       </c>
       <c r="Q2" s="2" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="R2" s="2" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="S2" s="5" t="s">
-        <v>106</v>
+        <v>91</v>
       </c>
       <c r="T2" s="2" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="U2" s="5" t="s">
-        <v>108</v>
+        <v>93</v>
       </c>
       <c r="V2" s="5" t="s">
-        <v>110</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>103</v>
+        <v>88</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>56</v>
+        <v>328</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>339</v>
+        <v>323</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>46</v>
+        <v>331</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>57</v>
+        <v>334</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>105</v>
+        <v>90</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>60</v>
+        <v>341</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>51</v>
+        <v>344</v>
       </c>
       <c r="L3" s="3">
         <v>32643</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>62</v>
+        <v>338</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>88</v>
+        <v>73</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>107</v>
+        <v>92</v>
       </c>
       <c r="T3" s="2" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>109</v>
+        <v>94</v>
       </c>
       <c r="V3" s="5" t="s">
-        <v>111</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>112</v>
+        <v>97</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>67</v>
+        <v>329</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>340</v>
+        <v>324</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>68</v>
+        <v>332</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>69</v>
+        <v>335</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>114</v>
+        <v>99</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>116</v>
+        <v>101</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>72</v>
+        <v>342</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>51</v>
+        <v>344</v>
       </c>
       <c r="L4" s="3">
         <v>33846</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>74</v>
+        <v>199</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="P4" s="2" t="s">
-        <v>87</v>
+        <v>72</v>
       </c>
       <c r="Q4" s="2" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="R4" s="2" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="S4" s="5" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="T4" s="2" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="U4" s="5" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="V4" s="5" t="s">
-        <v>122</v>
+        <v>107</v>
       </c>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>113</v>
+        <v>98</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>78</v>
+        <v>330</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>342</v>
+        <v>326</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>46</v>
+        <v>331</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>79</v>
+        <v>336</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>80</v>
+        <v>66</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>81</v>
+        <v>67</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>82</v>
+        <v>343</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>51</v>
+        <v>344</v>
       </c>
       <c r="L5" s="3">
         <v>34800</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>83</v>
+        <v>68</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>84</v>
+        <v>339</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>85</v>
+        <v>70</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="R5" s="2" t="s">
-        <v>84</v>
+        <v>69</v>
       </c>
       <c r="S5" s="5" t="s">
-        <v>119</v>
+        <v>104</v>
       </c>
       <c r="T5" s="2" t="s">
-        <v>91</v>
+        <v>76</v>
       </c>
       <c r="U5" s="5" t="s">
-        <v>121</v>
+        <v>106</v>
       </c>
       <c r="V5" s="5" t="s">
-        <v>123</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -2328,453 +2337,453 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>337</v>
+        <v>321</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>237</v>
+        <v>221</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>238</v>
+        <v>222</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>239</v>
+        <v>223</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>240</v>
+        <v>224</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>241</v>
+        <v>225</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>242</v>
+        <v>226</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>243</v>
+        <v>227</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>244</v>
+        <v>228</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>245</v>
+        <v>229</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>246</v>
+        <v>230</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>247</v>
+        <v>231</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>248</v>
+        <v>232</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>102</v>
+        <v>87</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="L2" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>206</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>212</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>266</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="L2" s="5" t="s">
-        <v>221</v>
-      </c>
       <c r="M2" s="2" t="s">
-        <v>211</v>
+        <v>195</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>103</v>
+        <v>88</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>213</v>
+        <v>197</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>214</v>
+        <v>198</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>217</v>
+        <v>201</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>218</v>
+        <v>202</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>219</v>
+        <v>203</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>267</v>
+        <v>251</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>271</v>
+        <v>255</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>223</v>
+        <v>207</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>236</v>
+        <v>220</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>222</v>
+        <v>206</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>224</v>
+        <v>208</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>112</v>
+        <v>97</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>225</v>
+        <v>209</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>226</v>
+        <v>210</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>227</v>
+        <v>211</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>228</v>
+        <v>212</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>229</v>
+        <v>213</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>230</v>
+        <v>214</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>268</v>
+        <v>252</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>231</v>
+        <v>215</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>232</v>
+        <v>216</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>233</v>
+        <v>217</v>
       </c>
       <c r="L4" s="5" t="s">
-        <v>234</v>
+        <v>218</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>235</v>
+        <v>219</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>113</v>
+        <v>98</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>249</v>
+        <v>233</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>250</v>
+        <v>234</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>251</v>
+        <v>235</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>252</v>
+        <v>236</v>
       </c>
       <c r="F5" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="H5" s="7" t="s">
         <v>253</v>
       </c>
-      <c r="G5" s="6" t="s">
-        <v>264</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>269</v>
-      </c>
       <c r="I5" s="7" t="s">
-        <v>254</v>
+        <v>238</v>
       </c>
       <c r="J5" s="7" t="s">
-        <v>255</v>
+        <v>239</v>
       </c>
       <c r="K5" s="7" t="s">
-        <v>256</v>
+        <v>240</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>257</v>
+        <v>241</v>
       </c>
       <c r="M5" s="7" t="s">
-        <v>258</v>
+        <v>242</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>180</v>
+        <v>164</v>
       </c>
       <c r="B6" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>247</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>249</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>254</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>256</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>257</v>
+      </c>
+      <c r="K6" s="7" t="s">
+        <v>258</v>
+      </c>
+      <c r="L6" s="6" t="s">
         <v>259</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="M6" s="7" t="s">
         <v>260</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>261</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>262</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>263</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>265</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>270</v>
-      </c>
-      <c r="I6" s="7" t="s">
-        <v>272</v>
-      </c>
-      <c r="J6" s="7" t="s">
-        <v>273</v>
-      </c>
-      <c r="K6" s="7" t="s">
-        <v>274</v>
-      </c>
-      <c r="L6" s="6" t="s">
-        <v>275</v>
-      </c>
-      <c r="M6" s="7" t="s">
-        <v>276</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>190</v>
+        <v>174</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>277</v>
+        <v>261</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>278</v>
+        <v>262</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>279</v>
+        <v>263</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>280</v>
+        <v>264</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>281</v>
+        <v>265</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>282</v>
+        <v>266</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>283</v>
+        <v>267</v>
       </c>
       <c r="I7" s="7" t="s">
+        <v>268</v>
+      </c>
+      <c r="J7" s="7" t="s">
+        <v>269</v>
+      </c>
+      <c r="K7" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="L7" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="M7" s="7" t="s">
         <v>284</v>
-      </c>
-      <c r="J7" s="7" t="s">
-        <v>285</v>
-      </c>
-      <c r="K7" s="7" t="s">
-        <v>286</v>
-      </c>
-      <c r="L7" s="6" t="s">
-        <v>287</v>
-      </c>
-      <c r="M7" s="7" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>194</v>
+        <v>178</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>288</v>
+        <v>272</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>289</v>
+        <v>273</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>290</v>
+        <v>274</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>291</v>
+        <v>275</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>292</v>
+        <v>276</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>293</v>
+        <v>277</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>294</v>
+        <v>278</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>295</v>
+        <v>279</v>
       </c>
       <c r="J8" s="7" t="s">
-        <v>296</v>
+        <v>280</v>
       </c>
       <c r="K8" s="7" t="s">
-        <v>297</v>
+        <v>281</v>
       </c>
       <c r="L8" s="6" t="s">
-        <v>298</v>
+        <v>282</v>
       </c>
       <c r="M8" s="7" t="s">
-        <v>299</v>
+        <v>283</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>198</v>
+        <v>182</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>302</v>
+        <v>286</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>303</v>
+        <v>287</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>304</v>
+        <v>288</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>305</v>
+        <v>289</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>306</v>
+        <v>290</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>307</v>
+        <v>291</v>
       </c>
       <c r="I9" s="7" t="s">
-        <v>308</v>
+        <v>292</v>
       </c>
       <c r="J9" s="7" t="s">
-        <v>309</v>
+        <v>293</v>
       </c>
       <c r="K9" s="7" t="s">
-        <v>310</v>
+        <v>294</v>
       </c>
       <c r="L9" s="6" t="s">
-        <v>311</v>
+        <v>295</v>
       </c>
       <c r="M9" s="7" t="s">
-        <v>312</v>
+        <v>296</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>338</v>
+        <v>322</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>313</v>
+        <v>297</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>314</v>
+        <v>298</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>315</v>
+        <v>299</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>316</v>
+        <v>300</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>317</v>
+        <v>301</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>318</v>
+        <v>302</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>319</v>
+        <v>303</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>320</v>
+        <v>304</v>
       </c>
       <c r="J10" s="7" t="s">
-        <v>321</v>
+        <v>305</v>
       </c>
       <c r="K10" s="7" t="s">
-        <v>322</v>
+        <v>306</v>
       </c>
       <c r="L10" s="6" t="s">
-        <v>323</v>
+        <v>307</v>
       </c>
       <c r="M10" s="7" t="s">
-        <v>324</v>
+        <v>308</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>165</v>
+        <v>149</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>325</v>
+        <v>309</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>326</v>
+        <v>310</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>327</v>
+        <v>311</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>328</v>
+        <v>312</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>329</v>
+        <v>313</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>330</v>
+        <v>314</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>331</v>
+        <v>315</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>332</v>
+        <v>316</v>
       </c>
       <c r="J11" s="7" t="s">
-        <v>333</v>
+        <v>317</v>
       </c>
       <c r="K11" s="7" t="s">
-        <v>334</v>
+        <v>318</v>
       </c>
       <c r="L11" s="6" t="s">
-        <v>335</v>
+        <v>319</v>
       </c>
       <c r="M11" s="7" t="s">
-        <v>336</v>
+        <v>320</v>
       </c>
     </row>
   </sheetData>

</xml_diff>